<commit_message>
added saves, updated excel file
</commit_message>
<xml_diff>
--- a/Excel_File/AquaSphare.xlsx
+++ b/Excel_File/AquaSphare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{167C95B2-D4F4-7C4E-AC15-9845565D49EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC49298-A999-2444-9FBB-8B9B85418EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1340" yWindow="1020" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
@@ -674,20 +674,6 @@
   <dxfs count="62">
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -886,6 +872,20 @@
           <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1867,23 +1867,23 @@
     <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="12"/>
     <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="11"/>
     <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="6">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="5">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="4">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1892,13 +1892,13 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="1">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="0">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D3" s="7" cm="1">
         <f t="array" ref="D3">Tabelle38[Actual time]</f>
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E3" s="7" cm="1">
         <f t="array" ref="E3">Tabelle49[[Total Storypoints ]]</f>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="F3" s="7">
         <f>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</f>
-        <v>0.875</v>
+        <v>0.61764705882352944</v>
       </c>
       <c r="G3" s="7">
         <v>146</v>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>0.125</v>
+        <v>8.8235294117647065E-2</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>1000</v>
+        <v>1416.6666666666665</v>
       </c>
     </row>
   </sheetData>
@@ -3711,9 +3711,11 @@
       <c r="I10" s="8">
         <v>3</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="8">
+        <v>10</v>
+      </c>
       <c r="K10" s="19" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -3823,11 +3825,11 @@
       </c>
       <c r="B17" s="12">
         <f>SUM(Tabelle27[Time in Hours])</f>
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C17" s="12">
         <f>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</f>
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="12">
@@ -3836,7 +3838,7 @@
       </c>
       <c r="F17" s="12">
         <f>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</f>
-        <v>0.875</v>
+        <v>0.61764705882352944</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>

</xml_diff>